<commit_message>
validation, testing dataset  creation
</commit_message>
<xml_diff>
--- a/ages_table.xlsx
+++ b/ages_table.xlsx
@@ -616,52 +616,52 @@
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
-        <v>4063</v>
+        <v>4033</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>56.42857143</v>
+        <v>57</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
-        <v>4033</v>
+        <v>4005</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>57</v>
+        <v>57.14285714</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
-        <v>4005</v>
+        <v>4062</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>57.14285714</v>
+        <v>57.57142857</v>
       </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
-        <v>4062</v>
+        <v>4037</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>57.57142857</v>
+        <v>58</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
-        <v>4037</v>
+        <v>4017</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>58</v>
+        <v>58.14285714</v>
       </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
-        <v>4017</v>
+        <v>4070</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>58.14285714</v>
@@ -670,52 +670,52 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
-        <v>4070</v>
+        <v>4090</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>58.14285714</v>
+        <v>58.28571429</v>
       </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
-        <v>4090</v>
+        <v>4035</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>58.28571429</v>
+        <v>59.57142857</v>
       </c>
       <c r="E25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
-        <v>4035</v>
+        <v>4088</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>59.57142857</v>
+        <v>59.71428571</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
-        <v>4088</v>
+        <v>4101</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>59.71428571</v>
+        <v>61.85714286</v>
       </c>
       <c r="E27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
-        <v>4101</v>
+        <v>4000</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>61.85714286</v>
+        <v>62</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
-        <v>4000</v>
+        <v>4011</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>62</v>
@@ -724,7 +724,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
-        <v>4011</v>
+        <v>4058</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>62</v>
@@ -733,106 +733,106 @@
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
-        <v>4058</v>
+        <v>4012</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>62</v>
+        <v>62.14285714</v>
       </c>
       <c r="E31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="n">
-        <v>4012</v>
+        <v>4019</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>62.14285714</v>
+        <v>62.71428571</v>
       </c>
       <c r="E32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="n">
-        <v>4019</v>
+        <v>4099</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>62.71428571</v>
+        <v>63.71428571</v>
       </c>
       <c r="E33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
-        <v>4099</v>
+        <v>4018</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>63.71428571</v>
+        <v>63.85714286</v>
       </c>
       <c r="E34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
-        <v>4018</v>
+        <v>4039</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>63.85714286</v>
+        <v>64.42857143</v>
       </c>
       <c r="E35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
-        <v>4039</v>
+        <v>4021</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>64.42857143</v>
+        <v>64.57142857</v>
       </c>
       <c r="E36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="n">
-        <v>4021</v>
+        <v>4097</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>64.57142857</v>
+        <v>65.14285714</v>
       </c>
       <c r="E37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="n">
-        <v>4097</v>
+        <v>4027</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>65.14285714</v>
+        <v>69</v>
       </c>
       <c r="E38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="n">
-        <v>4027</v>
+        <v>4010</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>69</v>
+        <v>69.42857143</v>
       </c>
       <c r="E39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="n">
-        <v>4010</v>
+        <v>4029</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>69.42857143</v>
+        <v>69.57142857</v>
       </c>
       <c r="E40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="n">
-        <v>4029</v>
+        <v>4001</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>69.57142857</v>
+        <v>70.28571429</v>
       </c>
       <c r="E41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="n">
-        <v>4001</v>
+        <v>4049</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>70.28571429</v>
@@ -841,490 +841,489 @@
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="n">
-        <v>4049</v>
+        <v>4085</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>70.28571429</v>
+        <v>72.14285714</v>
       </c>
       <c r="E43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="n">
-        <v>4085</v>
+        <v>4028</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>72.14285714</v>
+        <v>72.28571429</v>
       </c>
       <c r="E44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="n">
-        <v>4028</v>
+        <v>4031</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>72.28571429</v>
+        <v>72.57142857</v>
       </c>
       <c r="E45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="n">
-        <v>4031</v>
+        <v>4119</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>72.57142857</v>
+        <v>73.57142857</v>
       </c>
       <c r="E46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="n">
-        <v>4119</v>
+        <v>4084</v>
       </c>
       <c r="B47" s="1" t="n">
-        <v>73.57142857</v>
+        <v>74.42857143</v>
       </c>
       <c r="E47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="n">
-        <v>4084</v>
+        <v>4032</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>74.42857143</v>
+        <v>74.71428571</v>
       </c>
       <c r="E48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="n">
-        <v>4032</v>
+        <v>4086</v>
       </c>
       <c r="B49" s="1" t="n">
-        <v>74.71428571</v>
-      </c>
-      <c r="E49" s="2"/>
+        <v>75.57142857</v>
+      </c>
+      <c r="C49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="n">
-        <v>4086</v>
+        <v>4056</v>
       </c>
       <c r="B50" s="1" t="n">
-        <v>75.57142857</v>
+        <v>76</v>
       </c>
       <c r="C50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="n">
-        <v>4056</v>
+        <v>4026</v>
       </c>
       <c r="B51" s="1" t="n">
-        <v>76</v>
+        <v>76.57142857</v>
       </c>
       <c r="C51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="n">
-        <v>4026</v>
+        <v>4109</v>
       </c>
       <c r="B52" s="1" t="n">
-        <v>76.57142857</v>
+        <v>77.14285714</v>
       </c>
       <c r="C52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="n">
-        <v>4109</v>
+        <v>4030</v>
       </c>
       <c r="B53" s="1" t="n">
-        <v>77.14285714</v>
-      </c>
-      <c r="C53" s="2"/>
+        <v>79.28571429</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="n">
-        <v>4030</v>
+        <v>4034</v>
       </c>
       <c r="B54" s="1" t="n">
-        <v>79.28571429</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="n">
-        <v>4034</v>
+        <v>4083</v>
       </c>
       <c r="B55" s="1" t="n">
-        <v>80</v>
+        <v>81.42857143</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="n">
-        <v>4083</v>
+        <v>4022</v>
       </c>
       <c r="B56" s="1" t="n">
-        <v>81.42857143</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="n">
-        <v>4022</v>
+        <v>4014</v>
       </c>
       <c r="B57" s="1" t="n">
-        <v>82</v>
+        <v>82.28571429</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="n">
-        <v>4014</v>
+        <v>4072</v>
       </c>
       <c r="B58" s="1" t="n">
-        <v>82.28571429</v>
+        <v>85.28571429</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="n">
-        <v>4072</v>
+        <v>4050</v>
       </c>
       <c r="B59" s="1" t="n">
-        <v>85.28571429</v>
+        <v>86.14285714</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="n">
-        <v>4050</v>
+        <v>4096</v>
       </c>
       <c r="B60" s="1" t="n">
-        <v>86.14285714</v>
+        <v>91</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="n">
-        <v>4096</v>
+        <v>4025</v>
       </c>
       <c r="B61" s="1" t="n">
-        <v>91</v>
+        <v>91.85714286</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="n">
-        <v>4025</v>
+        <v>4045</v>
       </c>
       <c r="B62" s="1" t="n">
-        <v>91.85714286</v>
+        <v>93</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="n">
-        <v>4045</v>
+        <v>4102</v>
       </c>
       <c r="B63" s="1" t="n">
-        <v>93</v>
+        <v>96.28571429</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="n">
-        <v>4102</v>
+        <v>4002</v>
       </c>
       <c r="B64" s="1" t="n">
-        <v>96.28571429</v>
+        <v>98.14285714</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="n">
-        <v>4002</v>
+        <v>4042</v>
       </c>
       <c r="B65" s="1" t="n">
-        <v>98.14285714</v>
+        <v>98.71428571</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="n">
-        <v>4042</v>
+        <v>4015</v>
       </c>
       <c r="B66" s="1" t="n">
-        <v>98.71428571</v>
+        <v>102.1428571</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="n">
-        <v>4015</v>
+        <v>4081</v>
       </c>
       <c r="B67" s="1" t="n">
-        <v>102.1428571</v>
+        <v>113.7142857</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="n">
-        <v>4081</v>
+        <v>4065</v>
       </c>
       <c r="B68" s="1" t="n">
-        <v>113.7142857</v>
+        <v>115.7142857</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="n">
-        <v>4065</v>
+        <v>4091</v>
       </c>
       <c r="B69" s="1" t="n">
-        <v>115.7142857</v>
+        <v>123.4285714</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="n">
-        <v>4091</v>
+        <v>4075</v>
       </c>
       <c r="B70" s="1" t="n">
-        <v>123.4285714</v>
+        <v>128</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="n">
-        <v>4075</v>
+        <v>4043</v>
       </c>
       <c r="B71" s="1" t="n">
-        <v>128</v>
+        <v>129.5714286</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="n">
-        <v>4043</v>
+        <v>4054</v>
       </c>
       <c r="B72" s="1" t="n">
-        <v>129.5714286</v>
+        <v>132.1428571</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="n">
-        <v>4054</v>
+        <v>4013</v>
       </c>
       <c r="B73" s="1" t="n">
-        <v>132.1428571</v>
+        <v>133.4285714</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="n">
-        <v>4013</v>
+        <v>4110</v>
       </c>
       <c r="B74" s="1" t="n">
-        <v>133.4285714</v>
+        <v>149.5714286</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="n">
-        <v>4110</v>
+        <v>4069</v>
       </c>
       <c r="B75" s="1" t="n">
-        <v>149.5714286</v>
+        <v>155</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="n">
-        <v>4069</v>
+        <v>4020</v>
       </c>
       <c r="B76" s="1" t="n">
-        <v>155</v>
+        <v>162.5714286</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="n">
-        <v>4020</v>
+        <v>4106</v>
       </c>
       <c r="B77" s="1" t="n">
-        <v>162.5714286</v>
+        <v>171</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="n">
-        <v>4106</v>
+        <v>4111</v>
       </c>
       <c r="B78" s="1" t="n">
-        <v>171</v>
+        <v>176.8571429</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="n">
-        <v>4111</v>
+        <v>4113</v>
       </c>
       <c r="B79" s="1" t="n">
-        <v>176.8571429</v>
+        <v>179.2857143</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="n">
-        <v>4113</v>
+        <v>4047</v>
       </c>
       <c r="B80" s="1" t="n">
-        <v>179.2857143</v>
+        <v>181.1428571</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="n">
-        <v>4047</v>
+        <v>4046</v>
       </c>
       <c r="B81" s="1" t="n">
-        <v>181.1428571</v>
+        <v>188.7142857</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="n">
-        <v>4046</v>
+        <v>4107</v>
       </c>
       <c r="B82" s="1" t="n">
-        <v>188.7142857</v>
+        <v>194.8571429</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
-        <v>4107</v>
+        <v>4108</v>
       </c>
       <c r="B83" s="1" t="n">
-        <v>194.8571429</v>
+        <v>197</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="n">
-        <v>4108</v>
+        <v>4112</v>
       </c>
       <c r="B84" s="1" t="n">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="n">
-        <v>4112</v>
+        <v>4076</v>
       </c>
       <c r="B85" s="1" t="n">
-        <v>220</v>
+        <v>221.1428571</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="n">
-        <v>4076</v>
+        <v>4116</v>
       </c>
       <c r="B86" s="1" t="n">
-        <v>221.1428571</v>
+        <v>247.8571429</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="n">
-        <v>4116</v>
+        <v>4120</v>
       </c>
       <c r="B87" s="1" t="n">
-        <v>247.8571429</v>
+        <v>276.2857143</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="n">
-        <v>4120</v>
+        <v>404</v>
       </c>
       <c r="B88" s="1" t="n">
-        <v>276.2857143</v>
+        <v>299.715</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="n">
-        <v>4104</v>
+        <v>4118</v>
       </c>
       <c r="B89" s="1" t="n">
-        <v>297.7142857</v>
+        <v>300.8571429</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="n">
-        <v>404</v>
+        <v>4067</v>
       </c>
       <c r="B90" s="1" t="n">
-        <v>299.715</v>
+        <v>303.8571429</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="n">
-        <v>4118</v>
+        <v>4117</v>
       </c>
       <c r="B91" s="1" t="n">
-        <v>300.8571429</v>
+        <v>323.8571429</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="n">
-        <v>4067</v>
+        <v>4115</v>
       </c>
       <c r="B92" s="1" t="n">
-        <v>303.8571429</v>
+        <v>347</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="n">
-        <v>4117</v>
+        <v>4114</v>
       </c>
       <c r="B93" s="1" t="n">
-        <v>323.8571429</v>
+        <v>347.7142857</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="n">
-        <v>4115</v>
+        <v>407</v>
       </c>
       <c r="B94" s="1" t="n">
-        <v>347</v>
+        <v>351.858</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="n">
-        <v>4114</v>
+        <v>422</v>
       </c>
       <c r="B95" s="1" t="n">
-        <v>347.7142857</v>
+        <v>404.001</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="n">
-        <v>407</v>
+        <v>424</v>
       </c>
       <c r="B96" s="1" t="n">
-        <v>351.858</v>
+        <v>404.001</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="n">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="B97" s="1" t="n">
-        <v>404.001</v>
+        <v>456.144</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="n">
-        <v>424</v>
+        <v>412</v>
       </c>
       <c r="B98" s="1" t="n">
-        <v>404.001</v>
+        <v>456.144</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="n">
-        <v>411</v>
+        <v>427</v>
       </c>
       <c r="B99" s="1" t="n">
-        <v>456.144</v>
+        <v>508.287</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="n">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="B100" s="1" t="n">
-        <v>456.144</v>
+        <v>560.43</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="n">
-        <v>427</v>
+        <v>409</v>
       </c>
       <c r="B101" s="1" t="n">
-        <v>508.287</v>
+        <v>560.43</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="n">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="B102" s="1" t="n">
         <v>560.43</v>
@@ -1332,7 +1331,7 @@
     </row>
     <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="n">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="B103" s="1" t="n">
         <v>560.43</v>
@@ -1340,23 +1339,23 @@
     </row>
     <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="n">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B104" s="1" t="n">
-        <v>560.43</v>
+        <v>612.573</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="n">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="B105" s="1" t="n">
-        <v>560.43</v>
+        <v>612.573</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="n">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B106" s="1" t="n">
         <v>612.573</v>
@@ -1364,7 +1363,7 @@
     </row>
     <row r="107" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="n">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="B107" s="1" t="n">
         <v>612.573</v>
@@ -1372,23 +1371,23 @@
     </row>
     <row r="108" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="n">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="B108" s="1" t="n">
-        <v>612.573</v>
+        <v>664.716</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="n">
-        <v>423</v>
+        <v>410</v>
       </c>
       <c r="B109" s="1" t="n">
-        <v>612.573</v>
+        <v>664.716</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="n">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="B110" s="1" t="n">
         <v>664.716</v>
@@ -1396,7 +1395,7 @@
     </row>
     <row r="111" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="n">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="B111" s="1" t="n">
         <v>664.716</v>
@@ -1404,7 +1403,7 @@
     </row>
     <row r="112" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="B112" s="1" t="n">
         <v>664.716</v>
@@ -1412,127 +1411,127 @@
     </row>
     <row r="113" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
-        <v>421</v>
+        <v>403</v>
       </c>
       <c r="B113" s="1" t="n">
-        <v>664.716</v>
+        <v>716.859</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="n">
-        <v>426</v>
+        <v>408</v>
       </c>
       <c r="B114" s="1" t="n">
-        <v>664.716</v>
+        <v>716.859</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="1" t="n">
-        <v>403</v>
+        <v>419</v>
       </c>
       <c r="B115" s="1" t="n">
-        <v>716.859</v>
+        <v>769.002</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="n">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B116" s="1" t="n">
-        <v>716.859</v>
+        <v>821.145</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="n">
-        <v>419</v>
+        <v>406</v>
       </c>
       <c r="B117" s="1" t="n">
-        <v>769.002</v>
+        <v>821.145</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="1" t="n">
-        <v>405</v>
+      <c r="A118" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="B118" s="1" t="n">
-        <v>821.145</v>
+        <v>926.38</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="1" t="n">
-        <v>406</v>
+      <c r="A119" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B119" s="1" t="n">
-        <v>821.145</v>
+        <v>926.38</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B120" s="1" t="n">
-        <v>926.38</v>
+        <v>1082.8</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B121" s="1" t="n">
-        <v>926.38</v>
+        <v>1291.36</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B122" s="1" t="n">
-        <v>1082.8</v>
+        <v>1395.64</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B123" s="1" t="n">
-        <v>1291.36</v>
+        <v>1499.92</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B124" s="1" t="n">
-        <v>1395.64</v>
+        <v>1525.99</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B125" s="1" t="n">
-        <v>1499.92</v>
+        <v>1552.06</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B126" s="1" t="n">
-        <v>1525.99</v>
+        <v>1708.48</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B127" s="1" t="n">
-        <v>1552.06</v>
+        <v>1708.48</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B128" s="1" t="n">
         <v>1708.48</v>
@@ -1540,7 +1539,7 @@
     </row>
     <row r="129" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B129" s="1" t="n">
         <v>1708.48</v>
@@ -1548,47 +1547,47 @@
     </row>
     <row r="130" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B130" s="1" t="n">
-        <v>1708.48</v>
+        <v>1812.76</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B131" s="1" t="n">
-        <v>1708.48</v>
+        <v>1864.9</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B132" s="1" t="n">
-        <v>1812.76</v>
+        <v>1864.9</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B133" s="1" t="n">
-        <v>1864.9</v>
+        <v>2021.32</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B134" s="1" t="n">
-        <v>1864.9</v>
+        <v>2021.32</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B135" s="1" t="n">
         <v>2021.32</v>
@@ -1596,7 +1595,7 @@
     </row>
     <row r="136" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B136" s="1" t="n">
         <v>2021.32</v>
@@ -1604,143 +1603,143 @@
     </row>
     <row r="137" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B137" s="1" t="n">
-        <v>2021.32</v>
+        <v>2073.46</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B138" s="1" t="n">
-        <v>2021.32</v>
+        <v>2073.46</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B139" s="1" t="n">
-        <v>2073.46</v>
+        <v>2125.6</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B140" s="1" t="n">
-        <v>2073.46</v>
+        <v>2177.74</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B141" s="1" t="n">
-        <v>2125.6</v>
+        <v>2229.88</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B142" s="1" t="n">
-        <v>2177.74</v>
+        <v>2386.3</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B143" s="1" t="n">
-        <v>2229.88</v>
+        <v>2438.44</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B144" s="1" t="n">
-        <v>2386.3</v>
+        <v>2699.14</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B145" s="1" t="n">
-        <v>2438.44</v>
+        <v>2803.42</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B146" s="1" t="n">
-        <v>2699.14</v>
+        <v>2907.7</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B147" s="1" t="n">
-        <v>2803.42</v>
+        <v>3116.26</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B148" s="1" t="n">
-        <v>2907.7</v>
+        <v>3220.54</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B149" s="1" t="n">
-        <v>3116.26</v>
+        <v>3272.68</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B150" s="1" t="n">
-        <v>3220.54</v>
+        <v>3324.82</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B151" s="1" t="n">
-        <v>3272.68</v>
+        <v>3324.82</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B152" s="1" t="n">
-        <v>3324.82</v>
+        <v>3376.96</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B153" s="1" t="n">
-        <v>3324.82</v>
+        <v>3376.96</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B154" s="1" t="n">
         <v>3376.96</v>
@@ -1748,39 +1747,39 @@
     </row>
     <row r="155" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B155" s="1" t="n">
-        <v>3376.96</v>
+        <v>3429.1</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B156" s="1" t="n">
-        <v>3376.96</v>
+        <v>3429.1</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B157" s="1" t="n">
-        <v>3429.1</v>
+        <v>3481.24</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B158" s="1" t="n">
-        <v>3429.1</v>
+        <v>3481.24</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B159" s="1" t="n">
         <v>3481.24</v>
@@ -1788,23 +1787,23 @@
     </row>
     <row r="160" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B160" s="1" t="n">
-        <v>3481.24</v>
+        <v>3533.38</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B161" s="1" t="n">
-        <v>3481.24</v>
+        <v>3533.38</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B162" s="1" t="n">
         <v>3533.38</v>
@@ -1812,23 +1811,23 @@
     </row>
     <row r="163" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B163" s="1" t="n">
-        <v>3533.38</v>
+        <v>3585.52</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B164" s="1" t="n">
-        <v>3533.38</v>
+        <v>3585.52</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B165" s="1" t="n">
         <v>3585.52</v>
@@ -1836,52 +1835,38 @@
     </row>
     <row r="166" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B166" s="1" t="n">
-        <v>3585.52</v>
+        <v>3689.8</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B167" s="1" t="n">
-        <v>3585.52</v>
+        <v>3794.08</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B168" s="1" t="n">
-        <v>3689.8</v>
+        <v>3846.22</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B169" s="1" t="n">
-        <v>3794.08</v>
-      </c>
-    </row>
-    <row r="170" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B170" s="1" t="n">
-        <v>3846.22</v>
-      </c>
-    </row>
-    <row r="171" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B171" s="1" t="n">
         <v>3898.36</v>
       </c>
     </row>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>